<commit_message>
Fase 3b parte 1: programa del PC de la administración
- sync/: publica cartera, informes y documentos desde C:\Aragon en linea\Para subir
  con las mismas validaciones del panel; avisos QUE CORREGIR y espera sin conexión.
- Instalador de doble clic (Python, librerías, clave secreta, tarea programada).
- Hoja Control en las plantillas de cartera e informe mensual.
- Manual del programa del PC y guía técnica.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantillas/ejemplo_cartera_PRUEBA.xlsx
+++ b/plantillas/ejemplo_cartera_PRUEBA.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Cartera" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Control" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +42,11 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +63,11 @@
         <fgColor rgb="00B7791F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -72,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -83,6 +92,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -465,6 +477,13 @@
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Total de la cartera para escribir al importar: 9234000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hoja Control (celdas amarillas): la llena la contadora con los totales del informe contable. La usa el programa del PC de la administración; en el panel, los totales se escriben a mano.</t>
         </is>
       </c>
     </row>
@@ -2385,4 +2404,62 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>dato</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>qué es</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>total_informe</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>9234000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Total de la cartera según el informe contable (en pesos, sin decimales)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Ejemplo con datos de prueba: el total coincide con la suma del archivo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>